<commit_message>
agrego función de audit para evaluar slackness --audit
</commit_message>
<xml_diff>
--- a/Dynamic_model/zenteno_parameters.xlsx
+++ b/Dynamic_model/zenteno_parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cltor\Documents\SB_Calibration_2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://conchaytoro365-my.sharepoint.com/personal/cristobal_torrealba_conchaytoro_cl/Documents/Documentos/Proyectos I+D/PI-4497/Resultados/2025/SB_Calibration_2025/Dynamic_model/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B175C98-77CA-4BD1-A3A0-86EA0CCEB32B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{708A1B0C-CE8A-4E9F-84D7-5F51B80A027D}"/>
+    <workbookView xWindow="22944" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{708A1B0C-CE8A-4E9F-84D7-5F51B80A027D}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Cristobal Torrealba:</t>
         </r>
@@ -56,7 +56,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 2025</t>
@@ -71,7 +71,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t>Cristobal Torrealba:</t>
         </r>
@@ -80,7 +80,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
-            <charset val="1"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 2025+2024</t>
@@ -158,14 +158,14 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -824,6 +824,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>